<commit_message>
feat: data de hoje permitida na criação + dois exemplos de planilha
- Validação de criação: data não pode ser ANTERIOR a hoje (hoje é permitido,
  é o limite). Antes exigia estritamente futura, o que barrava criar para hoje.
- /api/tarefas/modelo?tipo=completo|erros: dois exemplos
  (10 tarefas válidas | válidas + inválidas), via TipoPlanilhaExemplo
- exemplos/ regenerados (2 arquivos) pelo gerador oficial (fonte única no tool)
- Testes: "criar com data de hoje permite" + round-trip dos dois tipos (7 e 10 linhas)

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemplos/tarefas-exemplo.xlsx
+++ b/exemplos/tarefas-exemplo.xlsx
@@ -28,16 +28,19 @@
     <x:t>Prioridade</x:t>
   </x:si>
   <x:si>
-    <x:t>Preparar apresentação</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Slides do fechamento do trimestre</x:t>
+    <x:t>Preparar apresentação trimestral</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Slides e relatório de resultados</x:t>
   </x:si>
   <x:si>
     <x:t>Alta</x:t>
   </x:si>
   <x:si>
-    <x:t>Revisar Pull Request #128</x:t>
+    <x:t>Revisar contrato de prestação</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Cláusulas 3 e 7</x:t>
   </x:si>
   <x:si>
     <x:t>Média</x:t>
@@ -46,31 +49,49 @@
     <x:t>Comprar materiais de escritório</x:t>
   </x:si>
   <x:si>
-    <x:t>Canetas, papel e toner</x:t>
-  </x:si>
-  <x:si>
-    <x:t>baixa</x:t>
-  </x:si>
-  <x:si>
     <x:t/>
   </x:si>
   <x:si>
-    <x:t>Tarefa já vencida</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Prioridade desconhecida</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Urgente</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Data em formato inválido</x:t>
-  </x:si>
-  <x:si>
-    <x:t>data-invalida</x:t>
-  </x:si>
-  <x:si>
     <x:t>Baixa</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Reunião de alinhamento com cliente</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Definição de escopo</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Atualizar política de privacidade</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Adequação à LGPD</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Treinamento da equipe</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Onboarding dos novos membros</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Fechamento contábil mensal</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Backup dos sistemas</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Rotina trimestral</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Planejamento de marketing</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Campanha do segundo semestre</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Auditoria interna</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Processos financeiros</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -428,11 +449,11 @@
   <x:sheetPr>
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
-  <x:dimension ref="A1:D8"/>
+  <x:dimension ref="A1:D11"/>
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="29.282054" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="31.710625" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="33.710625" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="30.710625" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="19.139196" style="0" customWidth="1"/>
     <x:col min="4" max="4" width="10.139196" style="0" customWidth="1"/>
   </x:cols>
@@ -459,7 +480,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="C2" s="1">
-        <x:v>47848</x:v>
+        <x:v>47498</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
         <x:v>6</x:v>
@@ -469,33 +490,39 @@
       <x:c r="A3" s="0" t="s">
         <x:v>7</x:v>
       </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>8</x:v>
+      </x:c>
       <x:c r="C3" s="1">
-        <x:v>47848</x:v>
+        <x:v>47511</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:4">
       <x:c r="A4" s="0" t="s">
-        <x:v>9</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>10</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C4" s="1">
-        <x:v>47848</x:v>
+        <x:v>47524</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>11</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:4">
       <x:c r="A5" s="0" t="s">
-        <x:v>12</x:v>
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="B5" s="0" t="s">
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C5" s="1">
-        <x:v>47848</x:v>
+        <x:v>47536</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
         <x:v>6</x:v>
@@ -503,35 +530,86 @@
     </x:row>
     <x:row r="6" spans="1:4">
       <x:c r="A6" s="0" t="s">
-        <x:v>13</x:v>
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="B6" s="0" t="s">
+        <x:v>16</x:v>
       </x:c>
       <x:c r="C6" s="1">
-        <x:v>43831</x:v>
+        <x:v>47547</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:4">
       <x:c r="A7" s="0" t="s">
-        <x:v>14</x:v>
+        <x:v>17</x:v>
+      </x:c>
+      <x:c r="B7" s="0" t="s">
+        <x:v>18</x:v>
       </x:c>
       <x:c r="C7" s="1">
-        <x:v>47848</x:v>
+        <x:v>47561</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>15</x:v>
+        <x:v>12</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:4">
       <x:c r="A8" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="C8" s="0" t="s">
-        <x:v>17</x:v>
+        <x:v>19</x:v>
+      </x:c>
+      <x:c r="B8" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C8" s="1">
+        <x:v>47575</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>18</x:v>
+        <x:v>6</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" spans="1:4">
+      <x:c r="A9" s="0" t="s">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="B9" s="0" t="s">
+        <x:v>21</x:v>
+      </x:c>
+      <x:c r="C9" s="1">
+        <x:v>47589</x:v>
+      </x:c>
+      <x:c r="D9" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" spans="1:4">
+      <x:c r="A10" s="0" t="s">
+        <x:v>22</x:v>
+      </x:c>
+      <x:c r="B10" s="0" t="s">
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="C10" s="1">
+        <x:v>47611</x:v>
+      </x:c>
+      <x:c r="D10" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:4">
+      <x:c r="A11" s="0" t="s">
+        <x:v>24</x:v>
+      </x:c>
+      <x:c r="B11" s="0" t="s">
+        <x:v>25</x:v>
+      </x:c>
+      <x:c r="C11" s="1">
+        <x:v>47635</x:v>
+      </x:c>
+      <x:c r="D11" s="0" t="s">
+        <x:v>6</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>